<commit_message>
feat: Implement color rules feature for Excel data extraction
</commit_message>
<xml_diff>
--- a/public/sample-employees.xlsx
+++ b/public/sample-employees.xlsx
@@ -397,15 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,9 +413,12 @@
         <v>القسم</v>
       </c>
       <c r="E1" t="str">
+        <v>نوع التعيين</v>
+      </c>
+      <c r="F1" t="str">
         <v>تاريخ العمل</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>تاريخ التعيين</v>
       </c>
     </row>
@@ -432,19 +427,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>EMP-001</v>
+        <v>EMP001</v>
       </c>
       <c r="C2" t="str">
-        <v>محمد أحمد علي الحربي</v>
+        <v>أحمد محمد علي الزهراني</v>
       </c>
       <c r="D2" t="str">
         <v>الموارد البشرية</v>
       </c>
       <c r="E2" t="str">
-        <v>01/01/2020</v>
+        <v>دائم</v>
       </c>
       <c r="F2" t="str">
-        <v>15/12/2019</v>
+        <v>2018-03-15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2018-04-01</v>
       </c>
     </row>
     <row r="3">
@@ -452,19 +450,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>EMP-002</v>
+        <v>EMP002</v>
       </c>
       <c r="C3" t="str">
-        <v>سارة خالد محمد العتيبي</v>
+        <v>فاطمة سالم ناصر القحطاني</v>
       </c>
       <c r="D3" t="str">
-        <v>تقنية المعلومات</v>
+        <v>المحاسبة</v>
       </c>
       <c r="E3" t="str">
-        <v>15/03/2021</v>
+        <v>عقد</v>
       </c>
       <c r="F3" t="str">
-        <v>01/03/2021</v>
+        <v>2020-07-10</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2020-08-01</v>
       </c>
     </row>
     <row r="4">
@@ -472,19 +473,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>EMP-003</v>
+        <v>EMP003</v>
       </c>
       <c r="C4" t="str">
-        <v>عبدالله سعد ناصر القحطاني</v>
+        <v>خالد عبدالله يوسف الدوسري</v>
       </c>
       <c r="D4" t="str">
-        <v>المالية</v>
+        <v>تقنية المعلومات</v>
       </c>
       <c r="E4" t="str">
-        <v>01/06/2019</v>
+        <v>دائم</v>
       </c>
       <c r="F4" t="str">
-        <v>20/05/2019</v>
+        <v>2015-01-20</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2015-02-01</v>
       </c>
     </row>
     <row r="5">
@@ -492,19 +496,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>EMP-004</v>
+        <v>EMP004</v>
       </c>
       <c r="C5" t="str">
-        <v>نورة فهد سلمان الشمري</v>
+        <v>نورة إبراهيم حسن العتيبي</v>
       </c>
       <c r="D5" t="str">
-        <v>المشتريات</v>
+        <v>المبيعات</v>
       </c>
       <c r="E5" t="str">
-        <v>10/09/2022</v>
+        <v>مؤقت</v>
       </c>
       <c r="F5" t="str">
-        <v>01/09/2022</v>
+        <v>2022-11-05</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2022-11-15</v>
       </c>
     </row>
     <row r="6">
@@ -512,19 +519,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>EMP-005</v>
+        <v>EMP005</v>
       </c>
       <c r="C6" t="str">
-        <v>خالد عمر يوسف الدوسري</v>
+        <v>عمر سعد محمد الغامدي</v>
       </c>
       <c r="D6" t="str">
         <v>تقنية المعلومات</v>
       </c>
       <c r="E6" t="str">
-        <v>01/01/2018</v>
+        <v>عقد</v>
       </c>
       <c r="F6" t="str">
-        <v>15/12/2017</v>
+        <v>2019-06-01</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2019-07-01</v>
       </c>
     </row>
     <row r="7">
@@ -532,19 +542,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>EMP-006</v>
+        <v>EMP006</v>
       </c>
       <c r="C7" t="str">
-        <v>ريم ناصر عبدالعزيز الزهراني</v>
+        <v>منى عبدالرحمن فهد الشمري</v>
       </c>
       <c r="D7" t="str">
         <v>الموارد البشرية</v>
       </c>
       <c r="E7" t="str">
-        <v>05/05/2023</v>
+        <v>دائم</v>
       </c>
       <c r="F7" t="str">
-        <v>01/05/2023</v>
+        <v>2016-09-12</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2016-10-01</v>
       </c>
     </row>
     <row r="8">
@@ -552,19 +565,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>EMP-007</v>
+        <v>EMP007</v>
       </c>
       <c r="C8" t="str">
-        <v>أحمد محمد صالح المطيري</v>
+        <v>يوسف طارق نايف الحربي</v>
       </c>
       <c r="D8" t="str">
-        <v>المالية</v>
+        <v>المحاسبة</v>
       </c>
       <c r="E8" t="str">
-        <v>20/02/2020</v>
+        <v>مؤقت</v>
       </c>
       <c r="F8" t="str">
-        <v>10/02/2020</v>
+        <v>2023-02-20</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2023-03-01</v>
       </c>
     </row>
     <row r="9">
@@ -572,19 +588,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>EMP-008</v>
+        <v>EMP008</v>
       </c>
       <c r="C9" t="str">
-        <v>هند سعود فيصل الغامدي</v>
+        <v>ريم وليد جاسم الأنصاري</v>
       </c>
       <c r="D9" t="str">
-        <v>المشتريات</v>
+        <v>المبيعات</v>
       </c>
       <c r="E9" t="str">
-        <v>01/07/2021</v>
+        <v>دائم</v>
       </c>
       <c r="F9" t="str">
-        <v>20/06/2021</v>
+        <v>2017-05-08</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2017-06-01</v>
       </c>
     </row>
     <row r="10">
@@ -592,19 +611,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>EMP-009</v>
+        <v>EMP009</v>
       </c>
       <c r="C10" t="str">
-        <v>سلطان راشد عبدالله العنزي</v>
+        <v>بندر محمد عيسى السبيعي</v>
       </c>
       <c r="D10" t="str">
-        <v>العمليات</v>
+        <v>تقنية المعلومات</v>
       </c>
       <c r="E10" t="str">
-        <v>01/03/2017</v>
+        <v>متدرب</v>
       </c>
       <c r="F10" t="str">
-        <v>15/02/2017</v>
+        <v>2024-01-15</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2024-01-15</v>
       </c>
     </row>
     <row r="11">
@@ -612,24 +634,27 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>EMP-010</v>
+        <v>EMP010</v>
       </c>
       <c r="C11" t="str">
-        <v>منيرة حمد جاسم الرشيدي</v>
+        <v>هند عبدالعزيز سلطان المطيري</v>
       </c>
       <c r="D11" t="str">
-        <v>العمليات</v>
+        <v>الموارد البشرية</v>
       </c>
       <c r="E11" t="str">
-        <v>15/11/2022</v>
+        <v>عقد</v>
       </c>
       <c r="F11" t="str">
-        <v>01/11/2022</v>
+        <v>2021-04-03</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2021-05-01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>